<commit_message>
Add tank filter — train only on real vessels with heads + shells
Filters out 31 non-tank jobs (handrails, repair parts, nozzle sets, rolled
shells only, ladders) that were polluting training data with non-vessel
routing patterns.

Tank criteria: routing shows evidence of both head and shell via:
  - Head fab ops (.350, .355, .360, .365, .366, .450, .455, .460, .465, .466)
  - Shell fab ops (.300-.325) OR shell detail ops (.620, .725, .726)
  - OR assembly ops (.600, .640, .641, .645) that imply both exist

Results:
  - 418 tank jobs identified (from 449 total in Operations.csv)
  - Backtest mean error: 15.2% → 13.7%
  - Feature importance MAPE: 18.4% → 16.7%
  - Cleaner similarity matches (no more handrail-to-reactor confusions)

https://claude.ai/code/session_013xSi86q6f1xS9pA8MuzK5a
</commit_message>
<xml_diff>
--- a/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
+++ b/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
@@ -53,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,12 +78,6 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -103,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,7 +110,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +529,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>25-064, 25-066, 25-067, 25-059, 25-061</t>
+          <t>25-060, 25-067, 25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -714,7 +707,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -723,7 +716,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.20 (0.20-0.25)</t>
+          <t>ratio=0.25 (0.20-0.25)</t>
         </is>
       </c>
       <c r="I9" s="8" t="n"/>
@@ -751,7 +744,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -760,7 +753,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.42 (0.20-0.75)</t>
+          <t>ratio=0.50 (0.42-0.75)</t>
         </is>
       </c>
       <c r="I10" s="8" t="n"/>
@@ -788,7 +781,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
@@ -797,7 +790,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.33 (0.33-1.00)</t>
+          <t>ratio=1.00 (0.33-1.00)</t>
         </is>
       </c>
       <c r="I11" s="8" t="n"/>
@@ -834,7 +827,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.61-1.02)</t>
+          <t>ratio=0.88 (0.80-1.02)</t>
         </is>
       </c>
       <c r="I12" s="8" t="n"/>
@@ -879,7 +872,7 @@
         <v>40</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -888,7 +881,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.44 (0.33-0.50)</t>
+          <t>ratio=0.45 (0.33-0.67)</t>
         </is>
       </c>
       <c r="I14" s="8" t="n"/>
@@ -916,7 +909,7 @@
         <v>20</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -925,7 +918,7 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.45-0.72)</t>
+          <t>ratio=0.62 (0.45-0.72)</t>
         </is>
       </c>
       <c r="I15" s="8" t="n"/>
@@ -979,7 +972,7 @@
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.25 (1.12-1.50)</t>
+          <t>ratio=1.25 (1.00-1.50)</t>
         </is>
       </c>
       <c r="I17" s="8" t="n"/>
@@ -1070,7 +1063,7 @@
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.60-0.90)</t>
+          <t>ratio=0.68 (0.60-0.78)</t>
         </is>
       </c>
       <c r="I20" s="8" t="n"/>
@@ -1097,17 +1090,17 @@
       <c r="E21" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="10" t="n">
+      <c r="F21" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (n=2)</t>
+          <t>ratio=1.00 (1.00-1.00)</t>
         </is>
       </c>
       <c r="I21" s="8" t="n"/>
@@ -1222,7 +1215,7 @@
         <v>9</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -1231,7 +1224,7 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-0.94)</t>
+          <t>ratio=0.78 (0.50-0.94)</t>
         </is>
       </c>
       <c r="I25" s="8" t="n"/>
@@ -1259,7 +1252,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
@@ -1268,7 +1261,7 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.75 (0.25-0.83)</t>
+          <t>ratio=0.67 (0.25-0.75)</t>
         </is>
       </c>
       <c r="I26" s="8" t="n"/>
@@ -1296,7 +1289,7 @@
         <v>18</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
@@ -1305,7 +1298,7 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.56 (0.53-0.92)</t>
+          <t>ratio=0.53 (0.50-0.92)</t>
         </is>
       </c>
       <c r="I27" s="8" t="n"/>
@@ -1392,7 +1385,7 @@
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-4.00)</t>
+          <t>ratio=2.00 (2.00-3.00)</t>
         </is>
       </c>
       <c r="I30" s="8" t="n"/>
@@ -1466,7 +1459,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.00)</t>
+          <t>ratio=2.00 (2.00-3.00)</t>
         </is>
       </c>
       <c r="I32" s="8" t="n"/>
@@ -1494,7 +1487,7 @@
         <v>6</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -1503,7 +1496,7 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.33-1.00)</t>
+          <t>ratio=1.00 (0.33-1.08)</t>
         </is>
       </c>
       <c r="I33" s="8" t="n"/>
@@ -1557,7 +1550,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.50)</t>
+          <t>ratio=2.00 (1.00-3.00)</t>
         </is>
       </c>
       <c r="I35" s="8" t="n"/>
@@ -1631,7 +1624,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.50-1.00)</t>
+          <t>ratio=1.00 (1.00-1.00)</t>
         </is>
       </c>
       <c r="I37" s="8" t="n"/>
@@ -1750,7 +1743,7 @@
         <v>5</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
@@ -1759,7 +1752,7 @@
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.60-2.20)</t>
+          <t>ratio=1.60 (1.00-2.20)</t>
         </is>
       </c>
       <c r="I41" s="8" t="n"/>
@@ -1787,7 +1780,7 @@
         <v>8</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
@@ -1796,7 +1789,7 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.56-1.12)</t>
+          <t>ratio=0.69 (0.56-0.88)</t>
         </is>
       </c>
       <c r="I42" s="8" t="n"/>
@@ -1833,7 +1826,7 @@
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-1.00)</t>
+          <t>ratio=0.67 (0.50-1.17)</t>
         </is>
       </c>
       <c r="I43" s="8" t="n"/>
@@ -1861,7 +1854,7 @@
         <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
@@ -1870,7 +1863,7 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.92-1.00)</t>
+          <t>ratio=0.92 (0.75-1.00)</t>
         </is>
       </c>
       <c r="I44" s="8" t="n"/>
@@ -1985,7 +1978,7 @@
         <v>8</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
@@ -1994,7 +1987,7 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.12 (0.62-1.84)</t>
+          <t>ratio=1.62 (1.12-2.75)</t>
         </is>
       </c>
       <c r="I48" s="8" t="n"/>
@@ -2022,7 +2015,7 @@
         <v>18</v>
       </c>
       <c r="F49" s="9" t="n">
-        <v>16</v>
+        <v>19.5</v>
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
@@ -2031,7 +2024,7 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.89 (0.78-1.17)</t>
+          <t>ratio=1.08 (0.78-1.43)</t>
         </is>
       </c>
       <c r="I49" s="8" t="n"/>
@@ -2059,7 +2052,7 @@
         <v>6</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
@@ -2068,7 +2061,7 @@
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.75 (0.33-1.08)</t>
+          <t>ratio=1.00 (0.33-1.08)</t>
         </is>
       </c>
       <c r="I50" s="8" t="n"/>
@@ -2212,7 +2205,7 @@
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.33 (1.15-4.00)</t>
+          <t>ratio=1.33 (1.17-4.00)</t>
         </is>
       </c>
       <c r="I54" s="8" t="n"/>
@@ -2240,7 +2233,7 @@
         <v>20</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>41</v>
+        <v>46.8</v>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
@@ -2249,7 +2242,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.05 (1.05-2.80)</t>
+          <t>ratio=2.34 (1.49-3.17)</t>
         </is>
       </c>
       <c r="I55" s="8" t="n"/>
@@ -2286,7 +2279,7 @@
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.20-1.00)</t>
+          <t>ratio=1.00 (0.20-2.00)</t>
         </is>
       </c>
       <c r="I56" s="8" t="n"/>
@@ -2331,7 +2324,7 @@
         <v>48</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>53</v>
+        <v>50.5</v>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
@@ -2340,7 +2333,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.10 (0.91-1.40)</t>
+          <t>ratio=1.05 (0.69-1.40)</t>
         </is>
       </c>
       <c r="I58" s="8" t="n"/>
@@ -2377,7 +2370,7 @@
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.84 (0.52-0.91)</t>
+          <t>ratio=0.84 (0.72-0.91)</t>
         </is>
       </c>
       <c r="I59" s="8" t="n"/>
@@ -2442,7 +2435,7 @@
         <v>30</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>14.5</v>
+        <v>18</v>
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
@@ -2451,7 +2444,7 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.48 (0.37-1.19)</t>
+          <t>ratio=0.60 (0.37-1.19)</t>
         </is>
       </c>
       <c r="I61" s="8" t="n"/>
@@ -2516,7 +2509,7 @@
         <v>1</v>
       </c>
       <c r="F63" s="9" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
@@ -2525,7 +2518,7 @@
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-2.00)</t>
+          <t>ratio=1.25 (0.50-2.00)</t>
         </is>
       </c>
       <c r="I63" s="8" t="n"/>
@@ -2570,7 +2563,7 @@
         <v>1</v>
       </c>
       <c r="F65" s="9" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
@@ -2579,7 +2572,7 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>ratio=3.00 (1.00-5.00)</t>
+          <t>ratio=2.25 (1.00-5.00)</t>
         </is>
       </c>
       <c r="I65" s="8" t="n"/>
@@ -2760,7 +2753,7 @@
         <v>12</v>
       </c>
       <c r="F71" s="9" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
@@ -2769,7 +2762,7 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.21 (0.50-3.67)</t>
+          <t>ratio=1.08 (0.50-1.42)</t>
         </is>
       </c>
       <c r="I71" s="8" t="n"/>
@@ -2872,7 +2865,7 @@
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.25-2.25)</t>
+          <t>ratio=1.25 (0.25-3.38)</t>
         </is>
       </c>
       <c r="I74" s="8" t="n"/>
@@ -2983,7 +2976,7 @@
         <v>3</v>
       </c>
       <c r="F78" s="9" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
@@ -2992,7 +2985,7 @@
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.58 (1.33-2.00)</t>
+          <t>ratio=1.50 (1.33-2.00)</t>
         </is>
       </c>
       <c r="I78" s="8" t="n"/>
@@ -3062,7 +3055,7 @@
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-1.60)</t>
+          <t>ratio=1.50 (1.00-2.20)</t>
         </is>
       </c>
       <c r="I80" s="8" t="n"/>
@@ -3076,7 +3069,7 @@
         </is>
       </c>
       <c r="F82" s="1" t="n">
-        <v>412.8</v>
+        <v>430.5</v>
       </c>
     </row>
   </sheetData>
@@ -3144,7 +3137,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>25-064, 25-066, 25-067, 25-059, 25-061</t>
+          <t>25-060, 25-067, 25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -5116,35 +5109,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25-064</t>
+          <t>25-060</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25-066</t>
+          <t>25-067</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25-067</t>
+          <t>25-066</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25-059</t>
+          <t>25-061</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25-061</t>
+          <t>25-059</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5244,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5260,12 +5253,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ratio=0.20 (0.20-0.25)</t>
+          <t>ratio=0.25 (0.20-0.25)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5274,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5290,12 +5283,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ratio=0.42 (0.20-0.75)</t>
+          <t>ratio=0.50 (0.42-0.75)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5311,7 +5304,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5320,12 +5313,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ratio=0.33 (0.33-1.00)</t>
+          <t>ratio=1.00 (0.33-1.00)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5350,12 +5343,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.61-1.02)</t>
+          <t>ratio=0.88 (0.80-1.02)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5364,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5380,12 +5373,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ratio=0.44 (0.33-0.50)</t>
+          <t>ratio=0.45 (0.33-0.67)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5394,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5410,12 +5403,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.45-0.72)</t>
+          <t>ratio=0.62 (0.45-0.72)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5440,12 +5433,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ratio=1.25 (1.12-1.50)</t>
+          <t>ratio=1.25 (1.00-1.50)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5468,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5500,12 +5493,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.60-0.90)</t>
+          <t>ratio=0.68 (0.60-0.78)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5525,17 +5518,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ratio=1.00 (n=2)</t>
+          <t>ratio=1.00 (1.00-1.00)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>25-061, 25-059</t>
+          <t>25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5565,7 +5558,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5600,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -5616,12 +5609,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-0.94)</t>
+          <t>ratio=0.78 (0.50-0.94)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5630,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -5646,12 +5639,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ratio=0.75 (0.25-0.83)</t>
+          <t>ratio=0.67 (0.25-0.75)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5667,7 +5660,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -5676,12 +5669,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ratio=0.56 (0.53-0.92)</t>
+          <t>ratio=0.53 (0.50-0.92)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5732,12 +5725,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-4.00)</t>
+          <t>ratio=2.00 (2.00-3.00)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5760,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>25-064, 25-061, 25-059</t>
+          <t>25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5792,12 +5785,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.00)</t>
+          <t>ratio=2.00 (2.00-3.00)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>25-064, 25-061, 25-059</t>
+          <t>25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5806,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -5822,12 +5815,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.33-1.00)</t>
+          <t>ratio=1.00 (0.33-1.08)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>25-064, 25-061, 25-059</t>
+          <t>25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5878,12 +5871,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.50)</t>
+          <t>ratio=2.00 (1.00-3.00)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -5913,7 +5906,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>25-066, 25-064, 25-061, 25-059</t>
+          <t>25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -5938,12 +5931,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.50-1.00)</t>
+          <t>ratio=1.00 (1.00-1.00)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5966,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -6003,7 +5996,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6019,7 +6012,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -6028,12 +6021,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.60-2.20)</t>
+          <t>ratio=1.60 (1.00-2.20)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6042,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -6058,12 +6051,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.56-1.12)</t>
+          <t>ratio=0.69 (0.56-0.88)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6088,12 +6081,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-1.00)</t>
+          <t>ratio=0.67 (0.50-1.17)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6109,7 +6102,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -6118,12 +6111,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.92-1.00)</t>
+          <t>ratio=0.92 (0.75-1.00)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>25-064, 25-061, 25-059</t>
+          <t>25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6172,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6195,7 +6188,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -6204,12 +6197,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ratio=1.12 (0.62-1.84)</t>
+          <t>ratio=1.62 (1.12-2.75)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6218,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16</v>
+        <v>19.5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -6234,12 +6227,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ratio=0.89 (0.78-1.17)</t>
+          <t>ratio=1.08 (0.78-1.43)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6248,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -6264,12 +6257,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ratio=0.75 (0.33-1.08)</t>
+          <t>ratio=1.00 (0.33-1.08)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>25-066, 25-064, 25-061, 25-059</t>
+          <t>25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6292,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6355,7 +6348,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6380,12 +6373,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ratio=1.33 (1.15-4.00)</t>
+          <t>ratio=1.33 (1.17-4.00)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6394,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>41</v>
+        <v>46.8</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -6410,12 +6403,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ratio=2.05 (1.05-2.80)</t>
+          <t>ratio=2.34 (1.49-3.17)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6440,12 +6433,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.20-1.00)</t>
+          <t>ratio=1.00 (0.20-2.00)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6454,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>53</v>
+        <v>50.5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -6470,12 +6463,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ratio=1.10 (0.91-1.40)</t>
+          <t>ratio=1.05 (0.69-1.40)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6500,12 +6493,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ratio=0.84 (0.52-0.91)</t>
+          <t>ratio=0.84 (0.72-0.91)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6528,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6544,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>14.5</v>
+        <v>18</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -6560,12 +6553,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ratio=0.48 (0.37-1.19)</t>
+          <t>ratio=0.60 (0.37-1.19)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6588,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6604,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -6620,12 +6613,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-2.00)</t>
+          <t>ratio=1.25 (0.50-2.00)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>25-066, 25-064, 25-061, 25-059</t>
+          <t>25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6634,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -6650,12 +6643,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ratio=3.00 (1.00-5.00)</t>
+          <t>ratio=2.25 (1.00-5.00)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-059</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6772,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -6788,12 +6781,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ratio=1.21 (0.50-3.67)</t>
+          <t>ratio=1.08 (0.50-1.42)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6870,12 +6863,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.25-2.25)</t>
+          <t>ratio=1.25 (0.25-3.38)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>25-066, 25-064, 25-061, 25-059</t>
+          <t>25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -6943,7 +6936,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -6952,12 +6945,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ratio=1.58 (1.33-2.00)</t>
+          <t>ratio=1.50 (1.33-2.00)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
         </is>
       </c>
     </row>
@@ -7008,12 +7001,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-1.60)</t>
+          <t>ratio=1.50 (1.00-2.20)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-064, 25-061</t>
+          <t>25-067, 25-066, 25-061, 25-060</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-group hours prediction — beats human estimates
Replaces whole-job prediction with 12 independent gradient-boosted models,
one per operation group (NOZZLES, CUT_PREP, SHELLS, TOP_HEAD, etc.).
Each model uses the spec features most relevant to that group:
  - flange_count → NOZZLE hours (r=0.78)
  - plate_count → CUT_PREP hours (r=0.81)
  - max_plate_thickness → SHELLS hours (r=0.63)
  - Total_Price → FIT_ASSEMBLY hours (r=0.74)

Group-level predictions are distributed to individual operations using
historical within-group proportions.

Backtest results (20 completed tanks):
  Median error: 6.6% (vs 9.9% human estimates)
  Mean error: 12.3% (vs 12.4% human)
  Predictions beat estimates: 11/20 (55%)

https://claude.ai/code/session_013xSi86q6f1xS9pA8MuzK5a
</commit_message>
<xml_diff>
--- a/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
+++ b/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
@@ -53,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +78,12 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+        <bgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -97,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +116,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +536,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>25-060, 25-067, 25-066, 25-061, 25-059</t>
+          <t>25-059, 25-066, 25-067, 25-060, 25-064</t>
         </is>
       </c>
     </row>
@@ -624,12 +631,12 @@
       <c r="F6" s="8" t="n"/>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I6" s="8" t="n"/>
@@ -657,12 +664,12 @@
       <c r="F7" s="8" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I7" s="8" t="n"/>
@@ -707,7 +714,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>3</v>
+        <v>8.6</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -716,7 +723,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.25 (0.20-0.25)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="I9" s="8" t="n"/>
@@ -744,7 +751,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -753,7 +760,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.50 (0.42-0.75)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="I10" s="8" t="n"/>
@@ -781,7 +788,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
@@ -790,7 +797,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.00)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="I11" s="8" t="n"/>
@@ -818,7 +825,7 @@
         <v>30</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>26.5</v>
+        <v>4.2</v>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
@@ -827,7 +834,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.80-1.02)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="I12" s="8" t="n"/>
@@ -872,7 +879,7 @@
         <v>40</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>18</v>
+        <v>26.6</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -881,7 +888,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.45 (0.33-0.67)</t>
+          <t>group_total:33h</t>
         </is>
       </c>
       <c r="I14" s="8" t="n"/>
@@ -909,7 +916,7 @@
         <v>20</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>12.5</v>
+        <v>6.2</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -918,7 +925,7 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.62 (0.45-0.72)</t>
+          <t>group_total:33h</t>
         </is>
       </c>
       <c r="I15" s="8" t="n"/>
@@ -963,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>10</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -972,7 +979,7 @@
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.25 (1.00-1.50)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="I17" s="8" t="n"/>
@@ -1017,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -1026,7 +1033,7 @@
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="I19" s="8" t="n"/>
@@ -1054,7 +1061,7 @@
         <v>10</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>6.8</v>
+        <v>1.8</v>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
@@ -1063,7 +1070,7 @@
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.60-0.78)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="I20" s="8" t="n"/>
@@ -1091,7 +1098,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>2</v>
+        <v>5.5</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -1100,7 +1107,7 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="I21" s="8" t="n"/>
@@ -1145,7 +1152,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
@@ -1154,7 +1161,7 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.50-1.50)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I23" s="8" t="n"/>
@@ -1182,12 +1189,12 @@
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I24" s="8" t="n"/>
@@ -1215,7 +1222,7 @@
         <v>9</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>7</v>
+        <v>10.3</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -1224,7 +1231,7 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.78 (0.50-0.94)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I25" s="8" t="n"/>
@@ -1252,7 +1259,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>8</v>
+        <v>2.3</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
@@ -1261,7 +1268,7 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.25-0.75)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I26" s="8" t="n"/>
@@ -1298,7 +1305,7 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.53 (0.50-0.92)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I27" s="8" t="n"/>
@@ -1343,12 +1350,12 @@
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I29" s="8" t="n"/>
@@ -1376,7 +1383,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
@@ -1385,7 +1392,7 @@
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-3.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="I30" s="8" t="n"/>
@@ -1413,7 +1420,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
@@ -1422,7 +1429,7 @@
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="I31" s="8" t="n"/>
@@ -1450,7 +1457,7 @@
         <v>1</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
@@ -1459,7 +1466,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-3.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="I32" s="8" t="n"/>
@@ -1487,7 +1494,7 @@
         <v>6</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>6</v>
+        <v>4.4</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -1496,7 +1503,7 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.08)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="I33" s="8" t="n"/>
@@ -1541,7 +1548,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -1550,7 +1557,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="I35" s="8" t="n"/>
@@ -1578,7 +1585,7 @@
         <v>1</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -1587,7 +1594,7 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="I36" s="8" t="n"/>
@@ -1615,7 +1622,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -1624,7 +1631,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="I37" s="8" t="n"/>
@@ -1652,7 +1659,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
@@ -1661,7 +1668,7 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.50)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="I38" s="8" t="n"/>
@@ -1706,7 +1713,7 @@
         <v>5</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
@@ -1715,7 +1722,7 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.80 (0.60-1.00)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I40" s="8" t="n"/>
@@ -1743,7 +1750,7 @@
         <v>5</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>8</v>
+        <v>4.8</v>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
@@ -1752,7 +1759,7 @@
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.60 (1.00-2.20)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I41" s="8" t="n"/>
@@ -1780,7 +1787,7 @@
         <v>8</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>5.5</v>
+        <v>4.2</v>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
@@ -1789,7 +1796,7 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.69 (0.56-0.88)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I42" s="8" t="n"/>
@@ -1817,7 +1824,7 @@
         <v>3</v>
       </c>
       <c r="F43" s="9" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
@@ -1826,7 +1833,7 @@
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-1.17)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I43" s="8" t="n"/>
@@ -1854,7 +1861,7 @@
         <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
@@ -1863,7 +1870,7 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.92 (0.75-1.00)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="I44" s="8" t="n"/>
@@ -1908,12 +1915,12 @@
       <c r="F46" s="8" t="n"/>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I46" s="8" t="n"/>
@@ -1941,7 +1948,7 @@
         <v>4</v>
       </c>
       <c r="F47" s="9" t="n">
-        <v>4</v>
+        <v>23.7</v>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
@@ -1950,7 +1957,7 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.75-1.50)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I47" s="8" t="n"/>
@@ -1978,7 +1985,7 @@
         <v>8</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>13</v>
+        <v>13.8</v>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
@@ -1987,7 +1994,7 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.62 (1.12-2.75)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I48" s="8" t="n"/>
@@ -2015,7 +2022,7 @@
         <v>18</v>
       </c>
       <c r="F49" s="9" t="n">
-        <v>19.5</v>
+        <v>16.3</v>
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
@@ -2024,7 +2031,7 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.08 (0.78-1.43)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I49" s="8" t="n"/>
@@ -2052,7 +2059,7 @@
         <v>6</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>6</v>
+        <v>5.3</v>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
@@ -2061,7 +2068,7 @@
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.08)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I50" s="8" t="n"/>
@@ -2089,7 +2096,7 @@
         <v>36</v>
       </c>
       <c r="F51" s="9" t="n">
-        <v>16</v>
+        <v>9.6</v>
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
@@ -2098,7 +2105,7 @@
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.44 (0.22-1.59)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I51" s="8" t="n"/>
@@ -2126,12 +2133,12 @@
       <c r="F52" s="8" t="n"/>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I52" s="8" t="n"/>
@@ -2159,7 +2166,7 @@
         <v>5</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
@@ -2168,7 +2175,7 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.40 (0.80-1.80)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I53" s="8" t="n"/>
@@ -2196,7 +2203,7 @@
         <v>12</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>16</v>
+        <v>7.2</v>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
@@ -2205,7 +2212,7 @@
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.33 (1.17-4.00)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I54" s="8" t="n"/>
@@ -2233,7 +2240,7 @@
         <v>20</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>46.8</v>
+        <v>33</v>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
@@ -2242,7 +2249,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.34 (1.49-3.17)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="I55" s="8" t="n"/>
@@ -2269,17 +2276,17 @@
       <c r="E56" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F56" s="9" t="n">
+      <c r="F56" s="10" t="n">
         <v>3</v>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.20-2.00)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I56" s="8" t="n"/>
@@ -2324,7 +2331,7 @@
         <v>48</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>50.5</v>
+        <v>24.5</v>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
@@ -2333,7 +2340,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.05 (0.69-1.40)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I58" s="8" t="n"/>
@@ -2361,7 +2368,7 @@
         <v>32</v>
       </c>
       <c r="F59" s="9" t="n">
-        <v>27</v>
+        <v>30.5</v>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
@@ -2370,7 +2377,7 @@
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.84 (0.72-0.91)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I59" s="8" t="n"/>
@@ -2398,7 +2405,7 @@
         <v>8</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>7.5</v>
+        <v>15.2</v>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
@@ -2407,7 +2414,7 @@
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.94 (0.44-1.50)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I60" s="8" t="n"/>
@@ -2435,7 +2442,7 @@
         <v>30</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>18</v>
+        <v>30.3</v>
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
@@ -2444,7 +2451,7 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.60 (0.37-1.19)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I61" s="8" t="n"/>
@@ -2472,7 +2479,7 @@
         <v>5</v>
       </c>
       <c r="F62" s="9" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
@@ -2481,7 +2488,7 @@
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.80 (0.20-2.80)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I62" s="8" t="n"/>
@@ -2509,7 +2516,7 @@
         <v>1</v>
       </c>
       <c r="F63" s="9" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
@@ -2518,7 +2525,7 @@
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.50-2.00)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I63" s="8" t="n"/>
@@ -2563,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="F65" s="9" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
@@ -2572,7 +2579,7 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>ratio=2.25 (1.00-5.00)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="I65" s="8" t="n"/>
@@ -2600,12 +2607,12 @@
       <c r="F66" s="8" t="n"/>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I66" s="8" t="n"/>
@@ -2633,12 +2640,12 @@
       <c r="F67" s="8" t="n"/>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I67" s="8" t="n"/>
@@ -2666,12 +2673,12 @@
       <c r="F68" s="8" t="n"/>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I68" s="8" t="n"/>
@@ -2716,7 +2723,7 @@
         <v>2</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
@@ -2725,7 +2732,7 @@
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>ratio=0.50 (0.50-1.38)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="I70" s="8" t="n"/>
@@ -2753,7 +2760,7 @@
         <v>12</v>
       </c>
       <c r="F71" s="9" t="n">
-        <v>13</v>
+        <v>14.4</v>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
@@ -2762,7 +2769,7 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.08 (0.50-1.42)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="I71" s="8" t="n"/>
@@ -2790,12 +2797,12 @@
       <c r="F72" s="8" t="n"/>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I72" s="8" t="n"/>
@@ -2823,12 +2830,12 @@
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I73" s="8" t="n"/>
@@ -2856,7 +2863,7 @@
         <v>2</v>
       </c>
       <c r="F74" s="9" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
@@ -2865,7 +2872,7 @@
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.25-3.38)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="I74" s="8" t="n"/>
@@ -2893,12 +2900,12 @@
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I75" s="8" t="n"/>
@@ -2926,12 +2933,12 @@
       <c r="F76" s="8" t="n"/>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I76" s="8" t="n"/>
@@ -2976,7 +2983,7 @@
         <v>3</v>
       </c>
       <c r="F78" s="9" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
@@ -2985,7 +2992,7 @@
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.33-2.00)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="I78" s="8" t="n"/>
@@ -3013,12 +3020,12 @@
       <c r="F79" s="8" t="n"/>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
         <is>
-          <t>0h estimate</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I79" s="8" t="n"/>
@@ -3046,7 +3053,7 @@
         <v>5</v>
       </c>
       <c r="F80" s="9" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
@@ -3055,7 +3062,7 @@
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-2.20)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="I80" s="8" t="n"/>
@@ -3069,7 +3076,7 @@
         </is>
       </c>
       <c r="F82" s="1" t="n">
-        <v>430.5</v>
+        <v>416.3</v>
       </c>
     </row>
   </sheetData>
@@ -3137,7 +3144,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>25-060, 25-067, 25-066, 25-061, 25-059</t>
+          <t>25-059, 25-066, 25-067, 25-060, 25-064</t>
         </is>
       </c>
     </row>
@@ -5109,35 +5116,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25-060</t>
+          <t>25-059</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25-067</t>
+          <t>25-066</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25-066</t>
+          <t>25-067</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25-061</t>
+          <t>25-060</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25-059</t>
+          <t>25-064</t>
         </is>
       </c>
     </row>
@@ -5196,15 +5203,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5222,15 +5233,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5244,7 +5259,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>8.6</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5253,12 +5268,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ratio=0.25 (0.20-0.25)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(NOZZLES)</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5289,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5283,12 +5298,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ratio=0.50 (0.42-0.75)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(NOZZLES)</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5319,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5313,12 +5328,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.00)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(NOZZLES)</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5349,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26.5</v>
+        <v>4.2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5343,12 +5358,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ratio=0.88 (0.80-1.02)</t>
+          <t>group_total:34h</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(NOZZLES)</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5379,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>26.6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5373,12 +5388,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ratio=0.45 (0.33-0.67)</t>
+          <t>group_total:33h</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(CUT_PREP)</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5409,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>12.5</v>
+        <v>6.2</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5403,12 +5418,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ratio=0.62 (0.45-0.72)</t>
+          <t>group_total:33h</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(CUT_PREP)</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5439,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5433,12 +5448,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ratio=1.25 (1.00-1.50)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SUPPORTS)</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5469,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -5463,12 +5478,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(MISC_PARTS)</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5499,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.8</v>
+        <v>1.8</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -5493,12 +5508,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ratio=0.68 (0.60-0.78)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(MISC_PARTS)</t>
         </is>
       </c>
     </row>
@@ -5514,7 +5529,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>5.5</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -5523,12 +5538,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:10h</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>25-061, 25-060, 25-059</t>
+          <t>model(MISC_PARTS)</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5559,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -5553,12 +5568,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.50-1.50)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SHELLS)</t>
         </is>
       </c>
     </row>
@@ -5578,15 +5593,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5600,7 +5619,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>10.3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -5609,12 +5628,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ratio=0.78 (0.50-0.94)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SHELLS)</t>
         </is>
       </c>
     </row>
@@ -5630,7 +5649,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>8</v>
+        <v>2.3</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -5639,12 +5658,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.25-0.75)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SHELLS)</t>
         </is>
       </c>
     </row>
@@ -5669,12 +5688,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ratio=0.53 (0.50-0.92)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SHELLS)</t>
         </is>
       </c>
     </row>
@@ -5694,15 +5713,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5716,7 +5739,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -5725,12 +5748,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-3.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(TOP_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5746,7 +5769,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -5755,12 +5778,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>25-061, 25-060, 25-059</t>
+          <t>model(TOP_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5799,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -5785,12 +5808,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ratio=2.00 (2.00-3.00)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>25-061, 25-060, 25-059</t>
+          <t>model(TOP_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5806,7 +5829,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>4.4</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -5815,12 +5838,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.08)</t>
+          <t>group_total:9h</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>25-061, 25-060, 25-059</t>
+          <t>model(TOP_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5840,15 +5863,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5862,7 +5889,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -5871,12 +5898,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ratio=2.00 (1.00-3.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(BTM_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5892,7 +5919,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -5901,12 +5928,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>25-066, 25-061, 25-059</t>
+          <t>model(BTM_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5922,7 +5949,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -5931,12 +5958,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.00)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>model(BTM_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5979,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -5961,12 +5988,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ratio=1.00 (1.00-1.50)</t>
+          <t>group_total:6h</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>model(BTM_HEAD)</t>
         </is>
       </c>
     </row>
@@ -5982,7 +6009,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -5991,12 +6018,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ratio=0.80 (0.60-1.00)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SKIRT)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6039,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>8</v>
+        <v>4.8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -6021,12 +6048,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ratio=1.60 (1.00-2.20)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SKIRT)</t>
         </is>
       </c>
     </row>
@@ -6042,7 +6069,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5.5</v>
+        <v>4.2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -6051,12 +6078,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ratio=0.69 (0.56-0.88)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SKIRT)</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6099,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -6081,12 +6108,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ratio=0.67 (0.50-1.17)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(SKIRT)</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6129,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -6111,12 +6138,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ratio=0.92 (0.75-1.00)</t>
+          <t>group_total:22h</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>25-061, 25-060, 25-059</t>
+          <t>model(SKIRT)</t>
         </is>
       </c>
     </row>
@@ -6136,15 +6163,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6158,7 +6189,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>23.7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -6167,12 +6198,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.75-1.50)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6219,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>13</v>
+        <v>13.8</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -6197,12 +6228,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ratio=1.62 (1.12-2.75)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6249,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>19.5</v>
+        <v>16.3</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -6227,12 +6258,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ratio=1.08 (0.78-1.43)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6279,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>5.3</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -6257,12 +6288,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.33-1.08)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6278,7 +6309,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>16</v>
+        <v>9.6</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -6287,12 +6318,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ratio=0.44 (0.22-1.59)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6312,15 +6343,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6334,7 +6369,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -6343,12 +6378,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ratio=1.40 (0.80-1.80)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6399,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>16</v>
+        <v>7.2</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -6373,12 +6408,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ratio=1.33 (1.17-4.00)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6394,7 +6429,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>46.8</v>
+        <v>33</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -6403,12 +6438,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ratio=2.34 (1.49-3.17)</t>
+          <t>group_total:123h</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(FIT_ASSEMBLY)</t>
         </is>
       </c>
     </row>
@@ -6428,17 +6463,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ratio=1.00 (0.20-2.00)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>nan</t>
         </is>
       </c>
     </row>
@@ -6454,7 +6489,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>50.5</v>
+        <v>24.5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -6463,12 +6498,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ratio=1.05 (0.69-1.40)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6519,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>27</v>
+        <v>30.5</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -6493,12 +6528,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ratio=0.84 (0.72-0.91)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6549,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>7.5</v>
+        <v>15.2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -6523,12 +6558,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ratio=0.94 (0.44-1.50)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6544,7 +6579,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>18</v>
+        <v>30.3</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -6553,12 +6588,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ratio=0.60 (0.37-1.19)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6574,7 +6609,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -6583,12 +6618,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ratio=1.80 (0.20-2.80)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6604,7 +6639,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -6613,12 +6648,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.50-2.00)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>25-066, 25-061, 25-060, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6634,7 +6669,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -6643,12 +6678,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ratio=2.25 (1.00-5.00)</t>
+          <t>group_total:115h</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-059</t>
+          <t>model(DETAIL_EXT)</t>
         </is>
       </c>
     </row>
@@ -6668,15 +6703,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6694,15 +6733,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6720,15 +6763,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6742,7 +6789,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -6751,12 +6798,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ratio=0.50 (0.50-1.38)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>25-067, 25-061, 25-059</t>
+          <t>model(TEST_CLEAN)</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6819,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>13</v>
+        <v>14.4</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -6781,12 +6828,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ratio=1.08 (0.50-1.42)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(TEST_CLEAN)</t>
         </is>
       </c>
     </row>
@@ -6806,15 +6853,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6832,15 +6883,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6854,7 +6909,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -6863,12 +6918,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ratio=1.25 (0.25-3.38)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>25-066, 25-061, 25-060, 25-059</t>
+          <t>model(TEST_CLEAN)</t>
         </is>
       </c>
     </row>
@@ -6888,15 +6943,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6914,15 +6973,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6936,7 +6999,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -6945,12 +7008,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.33-2.00)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060, 25-059</t>
+          <t>model(TEST_CLEAN)</t>
         </is>
       </c>
     </row>
@@ -6970,15 +7033,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>none</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>0h estimate</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6992,7 +7059,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -7001,12 +7068,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ratio=1.50 (1.00-2.20)</t>
+          <t>group_total:29h</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>25-067, 25-066, 25-061, 25-060</t>
+          <t>model(TEST_CLEAN)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add plate dimension features from BOM — SHELLS R² jumps 3x
Extracts plate qty, width, thickness, and cost from material_reqs BOM
descriptions (e.g., "PLT 316L 1/4 X 60 X" → thickness=0.25", width=60").

Key new features:
  total_plate_qty (r=0.67 with actual hrs)
  n_plate_lines (r=0.69)
  n_distinct_thicknesses (r=0.69)
  avg_plate_thickness (r=0.48)

Per-group model improvements:
  SHELLS: R² 0.10 → 0.30 (3x)
  CUT_PREP: R² 0.63 → 0.71
  TEST_CLEAN: R² 0.41 → 0.55

Backtest: 12/20 beat human estimates (60%), mean error 12.2% vs 12.4% human

https://claude.ai/code/session_013xSi86q6f1xS9pA8MuzK5a
</commit_message>
<xml_diff>
--- a/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
+++ b/buildplan_generator/output/25-057 GENERATED BUILD PLAN.xlsx
@@ -879,7 +879,7 @@
         <v>40</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>26.6</v>
+        <v>26.2</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>group_total:33h</t>
+          <t>group_total:32h</t>
         </is>
       </c>
       <c r="I14" s="8" t="n"/>
@@ -916,7 +916,7 @@
         <v>20</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>group_total:33h</t>
+          <t>group_total:32h</t>
         </is>
       </c>
       <c r="I15" s="8" t="n"/>
@@ -970,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="I23" s="8" t="n"/>
@@ -1222,7 +1222,7 @@
         <v>9</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>10.3</v>
+        <v>10.9</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="I25" s="8" t="n"/>
@@ -1259,7 +1259,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="I26" s="8" t="n"/>
@@ -1296,7 +1296,7 @@
         <v>18</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="I27" s="8" t="n"/>
@@ -1383,7 +1383,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
@@ -1457,7 +1457,7 @@
         <v>1</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="I35" s="8" t="n"/>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="I36" s="8" t="n"/>
@@ -1622,7 +1622,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="I37" s="8" t="n"/>
@@ -1659,7 +1659,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="I38" s="8" t="n"/>
@@ -1861,7 +1861,7 @@
         <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         <v>4</v>
       </c>
       <c r="F47" s="9" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I47" s="8" t="n"/>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I48" s="8" t="n"/>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I49" s="8" t="n"/>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I50" s="8" t="n"/>
@@ -2096,7 +2096,7 @@
         <v>36</v>
       </c>
       <c r="F51" s="9" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I51" s="8" t="n"/>
@@ -2166,7 +2166,7 @@
         <v>5</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I53" s="8" t="n"/>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I54" s="8" t="n"/>
@@ -2240,7 +2240,7 @@
         <v>20</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>33</v>
+        <v>33.1</v>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="I55" s="8" t="n"/>
@@ -2331,7 +2331,7 @@
         <v>48</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I58" s="8" t="n"/>
@@ -2368,7 +2368,7 @@
         <v>32</v>
       </c>
       <c r="F59" s="9" t="n">
-        <v>30.5</v>
+        <v>30.7</v>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I59" s="8" t="n"/>
@@ -2405,7 +2405,7 @@
         <v>8</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>15.2</v>
+        <v>15.4</v>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I60" s="8" t="n"/>
@@ -2442,7 +2442,7 @@
         <v>30</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>30.3</v>
+        <v>30.5</v>
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I61" s="8" t="n"/>
@@ -2479,7 +2479,7 @@
         <v>5</v>
       </c>
       <c r="F62" s="9" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I62" s="8" t="n"/>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I63" s="8" t="n"/>
@@ -2570,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="F65" s="9" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="I65" s="8" t="n"/>
@@ -2723,7 +2723,7 @@
         <v>2</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="I70" s="8" t="n"/>
@@ -2760,7 +2760,7 @@
         <v>12</v>
       </c>
       <c r="F71" s="9" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="I71" s="8" t="n"/>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="I74" s="8" t="n"/>
@@ -2983,7 +2983,7 @@
         <v>3</v>
       </c>
       <c r="F78" s="9" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="I78" s="8" t="n"/>
@@ -3053,7 +3053,7 @@
         <v>5</v>
       </c>
       <c r="F80" s="9" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="I80" s="8" t="n"/>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="F82" s="1" t="n">
-        <v>416.3</v>
+        <v>417.9</v>
       </c>
     </row>
   </sheetData>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>26.6</v>
+        <v>26.2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>group_total:33h</t>
+          <t>group_total:32h</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5418,7 +5418,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>group_total:33h</t>
+          <t>group_total:32h</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -5439,7 +5439,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5529,7 +5529,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10.3</v>
+        <v>10.9</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -5628,7 +5628,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -5649,7 +5649,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -5679,7 +5679,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -5688,7 +5688,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>group_total:22h</t>
+          <t>group_total:24h</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5739,7 +5739,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5928,7 +5928,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5949,7 +5949,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>group_total:6h</t>
+          <t>group_total:5h</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -6189,7 +6189,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -6309,7 +6309,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -6318,7 +6318,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -6378,7 +6378,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>33</v>
+        <v>33.1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>group_total:123h</t>
+          <t>group_total:124h</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6489,7 +6489,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6519,7 +6519,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>30.5</v>
+        <v>30.7</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -6528,7 +6528,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6549,7 +6549,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>15.2</v>
+        <v>15.4</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -6558,7 +6558,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6579,7 +6579,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>30.3</v>
+        <v>30.5</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6609,7 +6609,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6648,7 +6648,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -6669,7 +6669,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>group_total:115h</t>
+          <t>group_total:116h</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -6789,7 +6789,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -6819,7 +6819,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -6999,7 +6999,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -7059,7 +7059,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -7068,7 +7068,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>group_total:29h</t>
+          <t>group_total:30h</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">

</xml_diff>